<commit_message>
edits and updates for clean code in data cleaning process
</commit_message>
<xml_diff>
--- a/data/case10_mask.xlsx
+++ b/data/case10_mask.xlsx
@@ -5260,7 +5260,7 @@
     </row>
     <row r="967">
       <c r="A967" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="968">
@@ -5270,7 +5270,7 @@
     </row>
     <row r="969">
       <c r="A969" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="970">
@@ -6590,7 +6590,7 @@
     </row>
     <row r="1233">
       <c r="A1233" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1234">
@@ -6620,7 +6620,7 @@
     </row>
     <row r="1239">
       <c r="A1239" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1240">
@@ -6705,12 +6705,12 @@
     </row>
     <row r="1256">
       <c r="A1256" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1257">
       <c r="A1257" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1258">
@@ -6720,12 +6720,12 @@
     </row>
     <row r="1259">
       <c r="A1259" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1260">
       <c r="A1260" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1261">
@@ -7310,7 +7310,7 @@
     </row>
     <row r="1377">
       <c r="A1377" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1378">
@@ -7320,7 +7320,7 @@
     </row>
     <row r="1379">
       <c r="A1379" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1380">
@@ -7330,7 +7330,7 @@
     </row>
     <row r="1381">
       <c r="A1381" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1382">
@@ -7345,7 +7345,7 @@
     </row>
     <row r="1384">
       <c r="A1384" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1385">
@@ -10975,7 +10975,7 @@
     </row>
     <row r="2110">
       <c r="A2110" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2111">
@@ -10995,7 +10995,7 @@
     </row>
     <row r="2114">
       <c r="A2114" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2115">
@@ -11015,7 +11015,7 @@
     </row>
     <row r="2118">
       <c r="A2118" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2119">
@@ -11035,7 +11035,7 @@
     </row>
     <row r="2122">
       <c r="A2122" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2123">
@@ -11540,7 +11540,7 @@
     </row>
     <row r="2223">
       <c r="A2223" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2224">
@@ -12840,7 +12840,7 @@
     </row>
     <row r="2483">
       <c r="A2483" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2484">
@@ -12890,7 +12890,7 @@
     </row>
     <row r="2493">
       <c r="A2493" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2494">
@@ -17240,7 +17240,7 @@
     </row>
     <row r="3363">
       <c r="A3363" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3364">
@@ -18360,7 +18360,7 @@
     </row>
     <row r="3587">
       <c r="A3587" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3588">
@@ -19230,7 +19230,7 @@
     </row>
     <row r="3761">
       <c r="A3761" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3762">
@@ -21545,7 +21545,7 @@
     </row>
     <row r="4224">
       <c r="A4224" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4225">
@@ -23235,7 +23235,7 @@
     </row>
     <row r="4562">
       <c r="A4562" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4563">
@@ -28965,17 +28965,17 @@
     </row>
     <row r="5708">
       <c r="A5708" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5709">
       <c r="A5709" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5710">
       <c r="A5710" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5711">
@@ -29765,7 +29765,7 @@
     </row>
     <row r="5868">
       <c r="A5868" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5869">
@@ -31615,17 +31615,17 @@
     </row>
     <row r="6238">
       <c r="A6238" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6239">
       <c r="A6239" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6240">
       <c r="A6240" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6241">
@@ -31640,12 +31640,12 @@
     </row>
     <row r="6243">
       <c r="A6243" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6244">
       <c r="A6244" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6245">
@@ -37095,7 +37095,7 @@
     </row>
     <row r="7334">
       <c r="A7334" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7335">
@@ -37495,7 +37495,7 @@
     </row>
     <row r="7414">
       <c r="A7414" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7415">
@@ -37555,7 +37555,7 @@
     </row>
     <row r="7426">
       <c r="A7426" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7427">
@@ -38080,17 +38080,17 @@
     </row>
     <row r="7531">
       <c r="A7531" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7532">
       <c r="A7532" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7533">
       <c r="A7533" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7534">
@@ -38430,7 +38430,7 @@
     </row>
     <row r="7601">
       <c r="A7601" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7602">
@@ -41865,17 +41865,17 @@
     </row>
     <row r="8288">
       <c r="A8288" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8289">
       <c r="A8289" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8290">
       <c r="A8290" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8291">
@@ -41895,7 +41895,7 @@
     </row>
     <row r="8294">
       <c r="A8294" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8295">
@@ -41930,7 +41930,7 @@
     </row>
     <row r="8301">
       <c r="A8301" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8302">
@@ -44165,7 +44165,7 @@
     </row>
     <row r="8748">
       <c r="A8748" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8749">
@@ -44180,7 +44180,7 @@
     </row>
     <row r="8751">
       <c r="A8751" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8752">
@@ -44285,22 +44285,22 @@
     </row>
     <row r="8772">
       <c r="A8772" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8773">
       <c r="A8773" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8774">
       <c r="A8774" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8775">
       <c r="A8775" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8776">
@@ -44310,22 +44310,22 @@
     </row>
     <row r="8777">
       <c r="A8777" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8778">
       <c r="A8778" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8779">
       <c r="A8779" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8780">
       <c r="A8780" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8781">
@@ -47070,7 +47070,7 @@
     </row>
     <row r="9329">
       <c r="A9329" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9330">
@@ -57025,7 +57025,7 @@
     </row>
     <row r="11320">
       <c r="A11320" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11321">
@@ -57035,7 +57035,7 @@
     </row>
     <row r="11322">
       <c r="A11322" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11323">
@@ -58625,7 +58625,7 @@
     </row>
     <row r="11640">
       <c r="A11640" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11641">
@@ -58710,7 +58710,7 @@
     </row>
     <row r="11657">
       <c r="A11657" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11658">
@@ -58725,22 +58725,22 @@
     </row>
     <row r="11660">
       <c r="A11660" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11661">
       <c r="A11661" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11662">
       <c r="A11662" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11663">
       <c r="A11663" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11664">
@@ -58750,12 +58750,12 @@
     </row>
     <row r="11665">
       <c r="A11665" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11666">
       <c r="A11666" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11667">
@@ -58765,17 +58765,17 @@
     </row>
     <row r="11668">
       <c r="A11668" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11669">
       <c r="A11669" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11670">
       <c r="A11670" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11671">
@@ -59995,12 +59995,12 @@
     </row>
     <row r="11914">
       <c r="A11914" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11915">
       <c r="A11915" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11916">
@@ -67385,7 +67385,7 @@
     </row>
     <row r="13392">
       <c r="A13392" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13393">
@@ -73540,12 +73540,12 @@
     </row>
     <row r="14623">
       <c r="A14623" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14624">
       <c r="A14624" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14625">
@@ -73835,7 +73835,7 @@
     </row>
     <row r="14682">
       <c r="A14682" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14683">
@@ -76755,7 +76755,7 @@
     </row>
     <row r="15266">
       <c r="A15266" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15267">
@@ -77855,7 +77855,7 @@
     </row>
     <row r="15486">
       <c r="A15486" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15487">
@@ -82275,7 +82275,7 @@
     </row>
     <row r="16370">
       <c r="A16370" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16371">
@@ -84900,22 +84900,22 @@
     </row>
     <row r="16895">
       <c r="A16895" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16896">
       <c r="A16896" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16897">
       <c r="A16897" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16898">
       <c r="A16898" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16899">
@@ -89835,7 +89835,7 @@
     </row>
     <row r="17882">
       <c r="A17882" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17883">
@@ -89845,7 +89845,7 @@
     </row>
     <row r="17884">
       <c r="A17884" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17885">
@@ -91680,7 +91680,7 @@
     </row>
     <row r="18251">
       <c r="A18251" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18252">
@@ -94580,7 +94580,7 @@
     </row>
     <row r="18831">
       <c r="A18831" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18832">
@@ -94605,7 +94605,7 @@
     </row>
     <row r="18836">
       <c r="A18836" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18837">
@@ -94625,7 +94625,7 @@
     </row>
     <row r="18840">
       <c r="A18840" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18841">
@@ -96600,7 +96600,7 @@
     </row>
     <row r="19235">
       <c r="A19235" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19236">
@@ -96625,7 +96625,7 @@
     </row>
     <row r="19240">
       <c r="A19240" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19241">
@@ -96645,7 +96645,7 @@
     </row>
     <row r="19244">
       <c r="A19244" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19245">
@@ -98215,7 +98215,7 @@
     </row>
     <row r="19558">
       <c r="A19558" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19559">
@@ -99025,7 +99025,7 @@
     </row>
     <row r="19720">
       <c r="A19720" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19721">
@@ -100715,17 +100715,17 @@
     </row>
     <row r="20058">
       <c r="A20058" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20059">
       <c r="A20059" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20060">
       <c r="A20060" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20061">
@@ -100740,12 +100740,12 @@
     </row>
     <row r="20063">
       <c r="A20063" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20064">
       <c r="A20064" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20065">
@@ -100760,7 +100760,7 @@
     </row>
     <row r="20067">
       <c r="A20067" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20068">
@@ -103140,12 +103140,12 @@
     </row>
     <row r="20543">
       <c r="A20543" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20544">
       <c r="A20544" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20545">
@@ -103155,17 +103155,17 @@
     </row>
     <row r="20546">
       <c r="A20546" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20547">
       <c r="A20547" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20548">
       <c r="A20548" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20549">
@@ -108980,7 +108980,7 @@
     </row>
     <row r="21711">
       <c r="A21711" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21712">
@@ -109385,22 +109385,22 @@
     </row>
     <row r="21792">
       <c r="A21792" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21793">
       <c r="A21793" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21794">
       <c r="A21794" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21795">
       <c r="A21795" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21796">
@@ -109820,7 +109820,7 @@
     </row>
     <row r="21879">
       <c r="A21879" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21880">

</xml_diff>